<commit_message>
weekly update: 追加 2026-07-20 周两店经营看板数据
基于全部订单口径更新营收/订单/复购，并同步天气与源表。

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/紫竹/紫竹-品类映射.xlsx
+++ b/data/紫竹/紫竹-品类映射.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="30">
   <si>
     <t>类目</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>主餐（意面、焗饭）</t>
+  </si>
+  <si>
+    <t>冰淇淋</t>
   </si>
 </sst>
 </file>
@@ -839,7 +842,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -862,6 +865,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1389,14 +1395,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="14.2307692307692" customWidth="1"/>
     <col min="2" max="2" width="24.3846153846154" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31" spans="1:2">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1570,6 +1576,14 @@
       </c>
       <c r="B22" s="3" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>